<commit_message>
fix(i18n): make English sample Excel parseable and add display aliases
</commit_message>
<xml_diff>
--- a/data/samples/en/step1-scenario-anchoring/english-credit-scenario-template.xlsx
+++ b/data/samples/en/step1-scenario-anchoring/english-credit-scenario-template.xlsx
@@ -413,164 +413,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>scenario</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Interview Direction</t>
+          <t>scenario_desc</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Method</t>
+          <t>sub_scenario</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Knowledge Type</t>
+          <t>sub_scenario_desc</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>interview_direction</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>method</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Anti-pattern</t>
+          <t>knowledge_type</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Experience Judgment</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>condition</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Exception</t>
+          <t>logic</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Source Doc</t>
+          <t>anti_pattern</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Source Location</t>
+          <t>experience_judgment</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>boundary</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Contributor</t>
+          <t>exception</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Evidence Count</t>
+          <t>source_doc</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Breakthrough Count</t>
+          <t>source_location</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>contributor</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>evidence_count</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>breakthrough_count</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>SME inclusive loan marketing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Marketing guide for SME inclusive loans</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>First-time customer credit grant</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>How to assess a first-time SME customer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Customer onboarding</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Risk identification criteria</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Verify both credit report and cash flow</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Decision Rule</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Credit Management Policy Chapter 3</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>New customer first credit grant</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Rating A and stable cash flow then approve</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Ignore cash flow and only look at collateral</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Credit Policy</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Chapter 2 3.1.2</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Expert A</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="T2" t="n">
         <v>3</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="U2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>